<commit_message>
docs: commit latest regenerated Excel test reports for selenium, appium and load testing
</commit_message>
<xml_diff>
--- a/appium-tests/Appium_Mobile_E2E_Test_Report.xlsx
+++ b/appium-tests/Appium_Mobile_E2E_Test_Report.xlsx
@@ -5502,7 +5502,7 @@
         <v>51</v>
       </c>
       <c r="I2" s="19">
-        <v>351</v>
+        <v>764</v>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -5531,7 +5531,7 @@
         <v>51</v>
       </c>
       <c r="I3" s="19">
-        <v>286</v>
+        <v>574</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -5560,7 +5560,7 @@
         <v>60</v>
       </c>
       <c r="I4" s="19">
-        <v>466</v>
+        <v>226</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -5589,7 +5589,7 @@
         <v>51</v>
       </c>
       <c r="I5" s="19">
-        <v>574</v>
+        <v>311</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -5618,7 +5618,7 @@
         <v>51</v>
       </c>
       <c r="I6" s="19">
-        <v>721</v>
+        <v>593</v>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -5647,7 +5647,7 @@
         <v>60</v>
       </c>
       <c r="I7" s="19">
-        <v>249</v>
+        <v>729</v>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -5676,7 +5676,7 @@
         <v>51</v>
       </c>
       <c r="I8" s="19">
-        <v>666</v>
+        <v>735</v>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -5705,7 +5705,7 @@
         <v>51</v>
       </c>
       <c r="I9" s="19">
-        <v>745</v>
+        <v>389</v>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -5734,7 +5734,7 @@
         <v>60</v>
       </c>
       <c r="I10" s="19">
-        <v>584</v>
+        <v>240</v>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -5763,7 +5763,7 @@
         <v>51</v>
       </c>
       <c r="I11" s="19">
-        <v>383</v>
+        <v>385</v>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -5792,7 +5792,7 @@
         <v>51</v>
       </c>
       <c r="I12" s="19">
-        <v>272</v>
+        <v>724</v>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -5821,7 +5821,7 @@
         <v>60</v>
       </c>
       <c r="I13" s="19">
-        <v>421</v>
+        <v>736</v>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -5850,7 +5850,7 @@
         <v>51</v>
       </c>
       <c r="I14" s="19">
-        <v>365</v>
+        <v>688</v>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -5879,7 +5879,7 @@
         <v>51</v>
       </c>
       <c r="I15" s="19">
-        <v>680</v>
+        <v>587</v>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -5908,7 +5908,7 @@
         <v>60</v>
       </c>
       <c r="I16" s="19">
-        <v>336</v>
+        <v>560</v>
       </c>
     </row>
     <row r="17" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -5937,7 +5937,7 @@
         <v>51</v>
       </c>
       <c r="I17" s="19">
-        <v>755</v>
+        <v>342</v>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -5966,7 +5966,7 @@
         <v>51</v>
       </c>
       <c r="I18" s="19">
-        <v>285</v>
+        <v>666</v>
       </c>
     </row>
     <row r="19" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -5995,7 +5995,7 @@
         <v>60</v>
       </c>
       <c r="I19" s="19">
-        <v>556</v>
+        <v>547</v>
       </c>
     </row>
     <row r="20" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -6024,7 +6024,7 @@
         <v>51</v>
       </c>
       <c r="I20" s="19">
-        <v>492</v>
+        <v>260</v>
       </c>
     </row>
     <row r="21" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -6053,7 +6053,7 @@
         <v>51</v>
       </c>
       <c r="I21" s="19">
-        <v>622</v>
+        <v>467</v>
       </c>
     </row>
     <row r="22" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -6082,7 +6082,7 @@
         <v>60</v>
       </c>
       <c r="I22" s="19">
-        <v>456</v>
+        <v>769</v>
       </c>
     </row>
     <row r="23" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -6111,7 +6111,7 @@
         <v>51</v>
       </c>
       <c r="I23" s="19">
-        <v>548</v>
+        <v>468</v>
       </c>
     </row>
     <row r="24" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -6140,7 +6140,7 @@
         <v>51</v>
       </c>
       <c r="I24" s="19">
-        <v>570</v>
+        <v>341</v>
       </c>
     </row>
     <row r="25" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -6169,7 +6169,7 @@
         <v>60</v>
       </c>
       <c r="I25" s="19">
-        <v>470</v>
+        <v>570</v>
       </c>
     </row>
     <row r="26" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -6198,7 +6198,7 @@
         <v>51</v>
       </c>
       <c r="I26" s="19">
-        <v>770</v>
+        <v>536</v>
       </c>
     </row>
     <row r="27" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -6227,7 +6227,7 @@
         <v>51</v>
       </c>
       <c r="I27" s="19">
-        <v>529</v>
+        <v>242</v>
       </c>
     </row>
     <row r="28" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -6256,7 +6256,7 @@
         <v>60</v>
       </c>
       <c r="I28" s="19">
-        <v>395</v>
+        <v>722</v>
       </c>
     </row>
     <row r="29" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -6285,7 +6285,7 @@
         <v>51</v>
       </c>
       <c r="I29" s="19">
-        <v>362</v>
+        <v>409</v>
       </c>
     </row>
     <row r="30" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -6314,7 +6314,7 @@
         <v>51</v>
       </c>
       <c r="I30" s="19">
-        <v>277</v>
+        <v>727</v>
       </c>
     </row>
     <row r="31" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -6343,7 +6343,7 @@
         <v>60</v>
       </c>
       <c r="I31" s="19">
-        <v>393</v>
+        <v>256</v>
       </c>
     </row>
     <row r="32" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -6372,7 +6372,7 @@
         <v>51</v>
       </c>
       <c r="I32" s="19">
-        <v>713</v>
+        <v>582</v>
       </c>
     </row>
     <row r="33" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -6401,7 +6401,7 @@
         <v>51</v>
       </c>
       <c r="I33" s="19">
-        <v>541</v>
+        <v>405</v>
       </c>
     </row>
     <row r="34" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -6430,7 +6430,7 @@
         <v>60</v>
       </c>
       <c r="I34" s="19">
-        <v>788</v>
+        <v>532</v>
       </c>
     </row>
     <row r="35" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -6459,7 +6459,7 @@
         <v>51</v>
       </c>
       <c r="I35" s="19">
-        <v>711</v>
+        <v>730</v>
       </c>
     </row>
     <row r="36" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -6488,7 +6488,7 @@
         <v>51</v>
       </c>
       <c r="I36" s="19">
-        <v>339</v>
+        <v>744</v>
       </c>
     </row>
     <row r="37" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -6517,7 +6517,7 @@
         <v>60</v>
       </c>
       <c r="I37" s="19">
-        <v>664</v>
+        <v>514</v>
       </c>
     </row>
     <row r="38" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -6546,7 +6546,7 @@
         <v>51</v>
       </c>
       <c r="I38" s="19">
-        <v>715</v>
+        <v>699</v>
       </c>
     </row>
     <row r="39" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -6575,7 +6575,7 @@
         <v>51</v>
       </c>
       <c r="I39" s="19">
-        <v>532</v>
+        <v>729</v>
       </c>
     </row>
     <row r="40" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -6604,7 +6604,7 @@
         <v>60</v>
       </c>
       <c r="I40" s="19">
-        <v>462</v>
+        <v>582</v>
       </c>
     </row>
     <row r="41" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -6633,7 +6633,7 @@
         <v>51</v>
       </c>
       <c r="I41" s="19">
-        <v>642</v>
+        <v>234</v>
       </c>
     </row>
     <row r="42" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -6662,7 +6662,7 @@
         <v>51</v>
       </c>
       <c r="I42" s="19">
-        <v>766</v>
+        <v>500</v>
       </c>
     </row>
     <row r="43" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -6691,7 +6691,7 @@
         <v>60</v>
       </c>
       <c r="I43" s="19">
-        <v>622</v>
+        <v>544</v>
       </c>
     </row>
     <row r="44" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -6720,7 +6720,7 @@
         <v>51</v>
       </c>
       <c r="I44" s="19">
-        <v>490</v>
+        <v>696</v>
       </c>
     </row>
     <row r="45" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -6749,7 +6749,7 @@
         <v>51</v>
       </c>
       <c r="I45" s="19">
-        <v>246</v>
+        <v>724</v>
       </c>
     </row>
     <row r="46" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -6778,7 +6778,7 @@
         <v>60</v>
       </c>
       <c r="I46" s="19">
-        <v>400</v>
+        <v>774</v>
       </c>
     </row>
     <row r="47" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -6807,7 +6807,7 @@
         <v>51</v>
       </c>
       <c r="I47" s="19">
-        <v>311</v>
+        <v>617</v>
       </c>
     </row>
     <row r="48" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -6836,7 +6836,7 @@
         <v>51</v>
       </c>
       <c r="I48" s="19">
-        <v>225</v>
+        <v>241</v>
       </c>
     </row>
     <row r="49" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -6865,7 +6865,7 @@
         <v>60</v>
       </c>
       <c r="I49" s="19">
-        <v>520</v>
+        <v>601</v>
       </c>
     </row>
     <row r="50" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -6894,7 +6894,7 @@
         <v>51</v>
       </c>
       <c r="I50" s="19">
-        <v>669</v>
+        <v>613</v>
       </c>
     </row>
     <row r="51" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -6923,7 +6923,7 @@
         <v>51</v>
       </c>
       <c r="I51" s="19">
-        <v>447</v>
+        <v>281</v>
       </c>
     </row>
     <row r="52" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -6952,7 +6952,7 @@
         <v>60</v>
       </c>
       <c r="I52" s="19">
-        <v>293</v>
+        <v>641</v>
       </c>
     </row>
     <row r="53" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -6981,7 +6981,7 @@
         <v>51</v>
       </c>
       <c r="I53" s="19">
-        <v>223</v>
+        <v>249</v>
       </c>
     </row>
     <row r="54" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -7010,7 +7010,7 @@
         <v>51</v>
       </c>
       <c r="I54" s="19">
-        <v>717</v>
+        <v>581</v>
       </c>
     </row>
     <row r="55" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -7039,7 +7039,7 @@
         <v>60</v>
       </c>
       <c r="I55" s="19">
-        <v>553</v>
+        <v>460</v>
       </c>
     </row>
     <row r="56" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -7068,7 +7068,7 @@
         <v>51</v>
       </c>
       <c r="I56" s="19">
-        <v>290</v>
+        <v>605</v>
       </c>
     </row>
     <row r="57" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -7097,7 +7097,7 @@
         <v>51</v>
       </c>
       <c r="I57" s="19">
-        <v>359</v>
+        <v>390</v>
       </c>
     </row>
     <row r="58" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -7126,7 +7126,7 @@
         <v>60</v>
       </c>
       <c r="I58" s="19">
-        <v>395</v>
+        <v>282</v>
       </c>
     </row>
     <row r="59" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -7155,7 +7155,7 @@
         <v>51</v>
       </c>
       <c r="I59" s="19">
-        <v>678</v>
+        <v>752</v>
       </c>
     </row>
     <row r="60" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -7184,7 +7184,7 @@
         <v>51</v>
       </c>
       <c r="I60" s="19">
-        <v>751</v>
+        <v>349</v>
       </c>
     </row>
     <row r="61" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -7213,7 +7213,7 @@
         <v>292</v>
       </c>
       <c r="I61" s="19">
-        <v>238</v>
+        <v>686</v>
       </c>
     </row>
     <row r="62" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -7242,7 +7242,7 @@
         <v>51</v>
       </c>
       <c r="I62" s="19">
-        <v>427</v>
+        <v>623</v>
       </c>
     </row>
     <row r="63" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -7271,7 +7271,7 @@
         <v>51</v>
       </c>
       <c r="I63" s="19">
-        <v>399</v>
+        <v>471</v>
       </c>
     </row>
     <row r="64" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -7300,7 +7300,7 @@
         <v>60</v>
       </c>
       <c r="I64" s="19">
-        <v>580</v>
+        <v>352</v>
       </c>
     </row>
     <row r="65" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -7329,7 +7329,7 @@
         <v>51</v>
       </c>
       <c r="I65" s="19">
-        <v>548</v>
+        <v>656</v>
       </c>
     </row>
     <row r="66" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -7358,7 +7358,7 @@
         <v>51</v>
       </c>
       <c r="I66" s="19">
-        <v>688</v>
+        <v>565</v>
       </c>
     </row>
     <row r="67" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -7387,7 +7387,7 @@
         <v>60</v>
       </c>
       <c r="I67" s="19">
-        <v>409</v>
+        <v>695</v>
       </c>
     </row>
     <row r="68" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -7416,7 +7416,7 @@
         <v>51</v>
       </c>
       <c r="I68" s="19">
-        <v>773</v>
+        <v>412</v>
       </c>
     </row>
     <row r="69" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -7445,7 +7445,7 @@
         <v>51</v>
       </c>
       <c r="I69" s="19">
-        <v>294</v>
+        <v>420</v>
       </c>
     </row>
     <row r="70" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -7474,7 +7474,7 @@
         <v>60</v>
       </c>
       <c r="I70" s="19">
-        <v>323</v>
+        <v>413</v>
       </c>
     </row>
     <row r="71" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -7503,7 +7503,7 @@
         <v>51</v>
       </c>
       <c r="I71" s="19">
-        <v>597</v>
+        <v>640</v>
       </c>
     </row>
     <row r="72" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -7532,7 +7532,7 @@
         <v>51</v>
       </c>
       <c r="I72" s="19">
-        <v>752</v>
+        <v>347</v>
       </c>
     </row>
     <row r="73" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -7561,7 +7561,7 @@
         <v>60</v>
       </c>
       <c r="I73" s="19">
-        <v>213</v>
+        <v>778</v>
       </c>
     </row>
     <row r="74" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -7590,7 +7590,7 @@
         <v>51</v>
       </c>
       <c r="I74" s="19">
-        <v>280</v>
+        <v>524</v>
       </c>
     </row>
     <row r="75" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -7619,7 +7619,7 @@
         <v>51</v>
       </c>
       <c r="I75" s="19">
-        <v>760</v>
+        <v>345</v>
       </c>
     </row>
     <row r="76" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -7648,7 +7648,7 @@
         <v>60</v>
       </c>
       <c r="I76" s="19">
-        <v>343</v>
+        <v>712</v>
       </c>
     </row>
     <row r="77" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -7677,7 +7677,7 @@
         <v>51</v>
       </c>
       <c r="I77" s="19">
-        <v>734</v>
+        <v>441</v>
       </c>
     </row>
     <row r="78" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -7706,7 +7706,7 @@
         <v>51</v>
       </c>
       <c r="I78" s="19">
-        <v>769</v>
+        <v>750</v>
       </c>
     </row>
     <row r="79" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -7735,7 +7735,7 @@
         <v>60</v>
       </c>
       <c r="I79" s="19">
-        <v>683</v>
+        <v>526</v>
       </c>
     </row>
     <row r="80" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -7764,7 +7764,7 @@
         <v>51</v>
       </c>
       <c r="I80" s="19">
-        <v>394</v>
+        <v>753</v>
       </c>
     </row>
     <row r="81" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -7793,7 +7793,7 @@
         <v>51</v>
       </c>
       <c r="I81" s="19">
-        <v>512</v>
+        <v>250</v>
       </c>
     </row>
     <row r="82" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -7822,7 +7822,7 @@
         <v>60</v>
       </c>
       <c r="I82" s="19">
-        <v>572</v>
+        <v>443</v>
       </c>
     </row>
     <row r="83" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -7851,7 +7851,7 @@
         <v>51</v>
       </c>
       <c r="I83" s="19">
-        <v>210</v>
+        <v>504</v>
       </c>
     </row>
     <row r="84" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -7880,7 +7880,7 @@
         <v>51</v>
       </c>
       <c r="I84" s="19">
-        <v>428</v>
+        <v>280</v>
       </c>
     </row>
     <row r="85" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -7909,7 +7909,7 @@
         <v>60</v>
       </c>
       <c r="I85" s="19">
-        <v>589</v>
+        <v>518</v>
       </c>
     </row>
     <row r="86" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -7938,7 +7938,7 @@
         <v>51</v>
       </c>
       <c r="I86" s="19">
-        <v>587</v>
+        <v>317</v>
       </c>
     </row>
     <row r="87" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -7967,7 +7967,7 @@
         <v>51</v>
       </c>
       <c r="I87" s="19">
-        <v>616</v>
+        <v>632</v>
       </c>
     </row>
     <row r="88" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -7996,7 +7996,7 @@
         <v>60</v>
       </c>
       <c r="I88" s="19">
-        <v>476</v>
+        <v>605</v>
       </c>
     </row>
     <row r="89" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -8025,7 +8025,7 @@
         <v>51</v>
       </c>
       <c r="I89" s="19">
-        <v>511</v>
+        <v>323</v>
       </c>
     </row>
     <row r="90" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -8054,7 +8054,7 @@
         <v>51</v>
       </c>
       <c r="I90" s="19">
-        <v>762</v>
+        <v>413</v>
       </c>
     </row>
     <row r="91" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -8083,7 +8083,7 @@
         <v>60</v>
       </c>
       <c r="I91" s="19">
-        <v>507</v>
+        <v>577</v>
       </c>
     </row>
     <row r="92" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -8112,7 +8112,7 @@
         <v>51</v>
       </c>
       <c r="I92" s="19">
-        <v>392</v>
+        <v>256</v>
       </c>
     </row>
     <row r="93" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -8141,7 +8141,7 @@
         <v>51</v>
       </c>
       <c r="I93" s="19">
-        <v>598</v>
+        <v>329</v>
       </c>
     </row>
     <row r="94" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -8170,7 +8170,7 @@
         <v>60</v>
       </c>
       <c r="I94" s="19">
-        <v>509</v>
+        <v>431</v>
       </c>
     </row>
     <row r="95" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -8199,7 +8199,7 @@
         <v>51</v>
       </c>
       <c r="I95" s="19">
-        <v>600</v>
+        <v>502</v>
       </c>
     </row>
     <row r="96" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -8228,7 +8228,7 @@
         <v>51</v>
       </c>
       <c r="I96" s="19">
-        <v>229</v>
+        <v>446</v>
       </c>
     </row>
     <row r="97" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -8257,7 +8257,7 @@
         <v>60</v>
       </c>
       <c r="I97" s="19">
-        <v>375</v>
+        <v>418</v>
       </c>
     </row>
     <row r="98" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -8286,7 +8286,7 @@
         <v>51</v>
       </c>
       <c r="I98" s="19">
-        <v>571</v>
+        <v>565</v>
       </c>
     </row>
     <row r="99" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -8315,7 +8315,7 @@
         <v>51</v>
       </c>
       <c r="I99" s="19">
-        <v>350</v>
+        <v>200</v>
       </c>
     </row>
     <row r="100" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -8344,7 +8344,7 @@
         <v>60</v>
       </c>
       <c r="I100" s="19">
-        <v>338</v>
+        <v>738</v>
       </c>
     </row>
     <row r="101" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -8373,7 +8373,7 @@
         <v>51</v>
       </c>
       <c r="I101" s="19">
-        <v>604</v>
+        <v>327</v>
       </c>
     </row>
     <row r="102" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -8402,7 +8402,7 @@
         <v>51</v>
       </c>
       <c r="I102" s="19">
-        <v>715</v>
+        <v>390</v>
       </c>
     </row>
     <row r="103" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -8431,7 +8431,7 @@
         <v>60</v>
       </c>
       <c r="I103" s="19">
-        <v>389</v>
+        <v>723</v>
       </c>
     </row>
     <row r="104" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -8460,7 +8460,7 @@
         <v>51</v>
       </c>
       <c r="I104" s="19">
-        <v>609</v>
+        <v>470</v>
       </c>
     </row>
     <row r="105" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -8489,7 +8489,7 @@
         <v>51</v>
       </c>
       <c r="I105" s="19">
-        <v>542</v>
+        <v>624</v>
       </c>
     </row>
     <row r="106" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -8518,7 +8518,7 @@
         <v>60</v>
       </c>
       <c r="I106" s="19">
-        <v>568</v>
+        <v>795</v>
       </c>
     </row>
     <row r="107" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -8547,7 +8547,7 @@
         <v>51</v>
       </c>
       <c r="I107" s="19">
-        <v>480</v>
+        <v>502</v>
       </c>
     </row>
     <row r="108" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -8576,7 +8576,7 @@
         <v>51</v>
       </c>
       <c r="I108" s="19">
-        <v>555</v>
+        <v>327</v>
       </c>
     </row>
     <row r="109" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -8605,7 +8605,7 @@
         <v>60</v>
       </c>
       <c r="I109" s="19">
-        <v>621</v>
+        <v>280</v>
       </c>
     </row>
     <row r="110" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -8634,7 +8634,7 @@
         <v>51</v>
       </c>
       <c r="I110" s="19">
-        <v>357</v>
+        <v>208</v>
       </c>
     </row>
     <row r="111" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -8663,7 +8663,7 @@
         <v>51</v>
       </c>
       <c r="I111" s="19">
-        <v>370</v>
+        <v>371</v>
       </c>
     </row>
     <row r="112" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -8692,7 +8692,7 @@
         <v>60</v>
       </c>
       <c r="I112" s="19">
-        <v>328</v>
+        <v>663</v>
       </c>
     </row>
     <row r="113" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -8721,7 +8721,7 @@
         <v>51</v>
       </c>
       <c r="I113" s="19">
-        <v>585</v>
+        <v>500</v>
       </c>
     </row>
     <row r="114" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -8750,7 +8750,7 @@
         <v>51</v>
       </c>
       <c r="I114" s="19">
-        <v>321</v>
+        <v>627</v>
       </c>
     </row>
     <row r="115" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -8779,7 +8779,7 @@
         <v>60</v>
       </c>
       <c r="I115" s="19">
-        <v>797</v>
+        <v>495</v>
       </c>
     </row>
     <row r="116" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -8808,7 +8808,7 @@
         <v>51</v>
       </c>
       <c r="I116" s="19">
-        <v>422</v>
+        <v>726</v>
       </c>
     </row>
     <row r="117" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -8837,7 +8837,7 @@
         <v>51</v>
       </c>
       <c r="I117" s="19">
-        <v>698</v>
+        <v>539</v>
       </c>
     </row>
     <row r="118" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -8866,7 +8866,7 @@
         <v>60</v>
       </c>
       <c r="I118" s="19">
-        <v>286</v>
+        <v>640</v>
       </c>
     </row>
     <row r="119" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -8895,7 +8895,7 @@
         <v>51</v>
       </c>
       <c r="I119" s="19">
-        <v>584</v>
+        <v>261</v>
       </c>
     </row>
     <row r="120" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -8924,7 +8924,7 @@
         <v>51</v>
       </c>
       <c r="I120" s="19">
-        <v>288</v>
+        <v>633</v>
       </c>
     </row>
     <row r="121" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -8953,7 +8953,7 @@
         <v>292</v>
       </c>
       <c r="I121" s="19">
-        <v>776</v>
+        <v>297</v>
       </c>
     </row>
     <row r="122" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -8982,7 +8982,7 @@
         <v>51</v>
       </c>
       <c r="I122" s="19">
-        <v>414</v>
+        <v>735</v>
       </c>
     </row>
     <row r="123" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -9011,7 +9011,7 @@
         <v>51</v>
       </c>
       <c r="I123" s="19">
-        <v>754</v>
+        <v>381</v>
       </c>
     </row>
     <row r="124" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -9040,7 +9040,7 @@
         <v>60</v>
       </c>
       <c r="I124" s="19">
-        <v>594</v>
+        <v>390</v>
       </c>
     </row>
     <row r="125" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -9069,7 +9069,7 @@
         <v>51</v>
       </c>
       <c r="I125" s="19">
-        <v>402</v>
+        <v>404</v>
       </c>
     </row>
     <row r="126" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -9098,7 +9098,7 @@
         <v>51</v>
       </c>
       <c r="I126" s="19">
-        <v>640</v>
+        <v>215</v>
       </c>
     </row>
     <row r="127" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -9127,7 +9127,7 @@
         <v>60</v>
       </c>
       <c r="I127" s="19">
-        <v>485</v>
+        <v>728</v>
       </c>
     </row>
     <row r="128" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -9156,7 +9156,7 @@
         <v>51</v>
       </c>
       <c r="I128" s="19">
-        <v>570</v>
+        <v>241</v>
       </c>
     </row>
     <row r="129" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -9185,7 +9185,7 @@
         <v>51</v>
       </c>
       <c r="I129" s="19">
-        <v>401</v>
+        <v>765</v>
       </c>
     </row>
     <row r="130" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -9214,7 +9214,7 @@
         <v>60</v>
       </c>
       <c r="I130" s="19">
-        <v>605</v>
+        <v>452</v>
       </c>
     </row>
     <row r="131" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -9243,7 +9243,7 @@
         <v>51</v>
       </c>
       <c r="I131" s="19">
-        <v>604</v>
+        <v>261</v>
       </c>
     </row>
     <row r="132" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -9272,7 +9272,7 @@
         <v>51</v>
       </c>
       <c r="I132" s="19">
-        <v>694</v>
+        <v>415</v>
       </c>
     </row>
     <row r="133" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -9301,7 +9301,7 @@
         <v>60</v>
       </c>
       <c r="I133" s="19">
-        <v>263</v>
+        <v>511</v>
       </c>
     </row>
     <row r="134" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -9330,7 +9330,7 @@
         <v>51</v>
       </c>
       <c r="I134" s="19">
-        <v>419</v>
+        <v>456</v>
       </c>
     </row>
     <row r="135" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -9359,7 +9359,7 @@
         <v>51</v>
       </c>
       <c r="I135" s="19">
-        <v>340</v>
+        <v>758</v>
       </c>
     </row>
     <row r="136" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -9388,7 +9388,7 @@
         <v>60</v>
       </c>
       <c r="I136" s="19">
-        <v>443</v>
+        <v>210</v>
       </c>
     </row>
     <row r="137" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -9417,7 +9417,7 @@
         <v>51</v>
       </c>
       <c r="I137" s="19">
-        <v>480</v>
+        <v>628</v>
       </c>
     </row>
     <row r="138" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -9446,7 +9446,7 @@
         <v>51</v>
       </c>
       <c r="I138" s="19">
-        <v>775</v>
+        <v>523</v>
       </c>
     </row>
     <row r="139" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -9475,7 +9475,7 @@
         <v>60</v>
       </c>
       <c r="I139" s="19">
-        <v>575</v>
+        <v>704</v>
       </c>
     </row>
     <row r="140" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -9504,7 +9504,7 @@
         <v>51</v>
       </c>
       <c r="I140" s="19">
-        <v>206</v>
+        <v>535</v>
       </c>
     </row>
     <row r="141" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -9533,7 +9533,7 @@
         <v>51</v>
       </c>
       <c r="I141" s="19">
-        <v>276</v>
+        <v>633</v>
       </c>
     </row>
     <row r="142" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -9562,7 +9562,7 @@
         <v>60</v>
       </c>
       <c r="I142" s="19">
-        <v>623</v>
+        <v>359</v>
       </c>
     </row>
     <row r="143" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -9591,7 +9591,7 @@
         <v>51</v>
       </c>
       <c r="I143" s="19">
-        <v>784</v>
+        <v>605</v>
       </c>
     </row>
     <row r="144" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -9620,7 +9620,7 @@
         <v>51</v>
       </c>
       <c r="I144" s="19">
-        <v>612</v>
+        <v>382</v>
       </c>
     </row>
     <row r="145" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -9649,7 +9649,7 @@
         <v>60</v>
       </c>
       <c r="I145" s="19">
-        <v>743</v>
+        <v>202</v>
       </c>
     </row>
     <row r="146" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -9678,7 +9678,7 @@
         <v>51</v>
       </c>
       <c r="I146" s="19">
-        <v>408</v>
+        <v>798</v>
       </c>
     </row>
     <row r="147" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -9707,7 +9707,7 @@
         <v>51</v>
       </c>
       <c r="I147" s="19">
-        <v>315</v>
+        <v>337</v>
       </c>
     </row>
     <row r="148" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -9736,7 +9736,7 @@
         <v>60</v>
       </c>
       <c r="I148" s="19">
-        <v>277</v>
+        <v>767</v>
       </c>
     </row>
     <row r="149" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -9765,7 +9765,7 @@
         <v>51</v>
       </c>
       <c r="I149" s="19">
-        <v>515</v>
+        <v>423</v>
       </c>
     </row>
     <row r="150" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -9794,7 +9794,7 @@
         <v>51</v>
       </c>
       <c r="I150" s="19">
-        <v>796</v>
+        <v>730</v>
       </c>
     </row>
     <row r="151" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -9823,7 +9823,7 @@
         <v>60</v>
       </c>
       <c r="I151" s="19">
-        <v>748</v>
+        <v>359</v>
       </c>
     </row>
     <row r="152" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -9852,7 +9852,7 @@
         <v>51</v>
       </c>
       <c r="I152" s="19">
-        <v>682</v>
+        <v>652</v>
       </c>
     </row>
     <row r="153" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -9881,7 +9881,7 @@
         <v>51</v>
       </c>
       <c r="I153" s="19">
-        <v>717</v>
+        <v>269</v>
       </c>
     </row>
     <row r="154" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -9910,7 +9910,7 @@
         <v>60</v>
       </c>
       <c r="I154" s="19">
-        <v>766</v>
+        <v>440</v>
       </c>
     </row>
     <row r="155" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -9939,7 +9939,7 @@
         <v>51</v>
       </c>
       <c r="I155" s="19">
-        <v>296</v>
+        <v>466</v>
       </c>
     </row>
     <row r="156" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -9968,7 +9968,7 @@
         <v>51</v>
       </c>
       <c r="I156" s="19">
-        <v>368</v>
+        <v>380</v>
       </c>
     </row>
     <row r="157" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -9997,7 +9997,7 @@
         <v>60</v>
       </c>
       <c r="I157" s="19">
-        <v>290</v>
+        <v>580</v>
       </c>
     </row>
     <row r="158" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -10026,7 +10026,7 @@
         <v>51</v>
       </c>
       <c r="I158" s="19">
-        <v>740</v>
+        <v>671</v>
       </c>
     </row>
     <row r="159" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -10055,7 +10055,7 @@
         <v>51</v>
       </c>
       <c r="I159" s="19">
-        <v>277</v>
+        <v>727</v>
       </c>
     </row>
     <row r="160" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -10084,7 +10084,7 @@
         <v>60</v>
       </c>
       <c r="I160" s="19">
-        <v>483</v>
+        <v>335</v>
       </c>
     </row>
     <row r="161" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -10113,7 +10113,7 @@
         <v>51</v>
       </c>
       <c r="I161" s="19">
-        <v>423</v>
+        <v>407</v>
       </c>
     </row>
     <row r="162" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -10142,7 +10142,7 @@
         <v>51</v>
       </c>
       <c r="I162" s="19">
-        <v>668</v>
+        <v>569</v>
       </c>
     </row>
     <row r="163" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -10171,7 +10171,7 @@
         <v>60</v>
       </c>
       <c r="I163" s="19">
-        <v>599</v>
+        <v>317</v>
       </c>
     </row>
     <row r="164" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -10200,7 +10200,7 @@
         <v>51</v>
       </c>
       <c r="I164" s="19">
-        <v>226</v>
+        <v>333</v>
       </c>
     </row>
     <row r="165" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -10229,7 +10229,7 @@
         <v>51</v>
       </c>
       <c r="I165" s="19">
-        <v>406</v>
+        <v>650</v>
       </c>
     </row>
     <row r="166" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -10258,7 +10258,7 @@
         <v>60</v>
       </c>
       <c r="I166" s="19">
-        <v>299</v>
+        <v>454</v>
       </c>
     </row>
     <row r="167" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -10287,7 +10287,7 @@
         <v>51</v>
       </c>
       <c r="I167" s="19">
-        <v>704</v>
+        <v>549</v>
       </c>
     </row>
     <row r="168" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -10316,7 +10316,7 @@
         <v>51</v>
       </c>
       <c r="I168" s="19">
-        <v>228</v>
+        <v>615</v>
       </c>
     </row>
     <row r="169" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -10345,7 +10345,7 @@
         <v>60</v>
       </c>
       <c r="I169" s="19">
-        <v>689</v>
+        <v>719</v>
       </c>
     </row>
     <row r="170" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -10374,7 +10374,7 @@
         <v>51</v>
       </c>
       <c r="I170" s="19">
-        <v>254</v>
+        <v>567</v>
       </c>
     </row>
     <row r="171" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -10403,7 +10403,7 @@
         <v>51</v>
       </c>
       <c r="I171" s="19">
-        <v>346</v>
+        <v>681</v>
       </c>
     </row>
     <row r="172" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -10432,7 +10432,7 @@
         <v>60</v>
       </c>
       <c r="I172" s="19">
-        <v>395</v>
+        <v>218</v>
       </c>
     </row>
     <row r="173" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -10461,7 +10461,7 @@
         <v>51</v>
       </c>
       <c r="I173" s="19">
-        <v>415</v>
+        <v>507</v>
       </c>
     </row>
     <row r="174" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -10490,7 +10490,7 @@
         <v>51</v>
       </c>
       <c r="I174" s="19">
-        <v>334</v>
+        <v>657</v>
       </c>
     </row>
     <row r="175" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -10519,7 +10519,7 @@
         <v>60</v>
       </c>
       <c r="I175" s="19">
-        <v>521</v>
+        <v>506</v>
       </c>
     </row>
     <row r="176" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -10548,7 +10548,7 @@
         <v>51</v>
       </c>
       <c r="I176" s="19">
-        <v>461</v>
+        <v>578</v>
       </c>
     </row>
     <row r="177" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -10577,7 +10577,7 @@
         <v>51</v>
       </c>
       <c r="I177" s="19">
-        <v>688</v>
+        <v>456</v>
       </c>
     </row>
     <row r="178" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -10606,7 +10606,7 @@
         <v>60</v>
       </c>
       <c r="I178" s="19">
-        <v>265</v>
+        <v>357</v>
       </c>
     </row>
     <row r="179" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -10635,7 +10635,7 @@
         <v>51</v>
       </c>
       <c r="I179" s="19">
-        <v>587</v>
+        <v>335</v>
       </c>
     </row>
     <row r="180" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -10664,7 +10664,7 @@
         <v>51</v>
       </c>
       <c r="I180" s="19">
-        <v>301</v>
+        <v>779</v>
       </c>
     </row>
     <row r="181" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -10693,7 +10693,7 @@
         <v>292</v>
       </c>
       <c r="I181" s="19">
-        <v>437</v>
+        <v>691</v>
       </c>
     </row>
     <row r="182" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -10722,7 +10722,7 @@
         <v>51</v>
       </c>
       <c r="I182" s="19">
-        <v>248</v>
+        <v>517</v>
       </c>
     </row>
     <row r="183" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -10751,7 +10751,7 @@
         <v>51</v>
       </c>
       <c r="I183" s="19">
-        <v>214</v>
+        <v>507</v>
       </c>
     </row>
     <row r="184" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -10780,7 +10780,7 @@
         <v>60</v>
       </c>
       <c r="I184" s="19">
-        <v>303</v>
+        <v>656</v>
       </c>
     </row>
     <row r="185" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -10809,7 +10809,7 @@
         <v>51</v>
       </c>
       <c r="I185" s="19">
-        <v>797</v>
+        <v>591</v>
       </c>
     </row>
     <row r="186" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -10838,7 +10838,7 @@
         <v>51</v>
       </c>
       <c r="I186" s="19">
-        <v>774</v>
+        <v>411</v>
       </c>
     </row>
     <row r="187" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -10867,7 +10867,7 @@
         <v>60</v>
       </c>
       <c r="I187" s="19">
-        <v>204</v>
+        <v>671</v>
       </c>
     </row>
     <row r="188" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -10896,7 +10896,7 @@
         <v>51</v>
       </c>
       <c r="I188" s="19">
-        <v>379</v>
+        <v>582</v>
       </c>
     </row>
     <row r="189" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -10925,7 +10925,7 @@
         <v>51</v>
       </c>
       <c r="I189" s="19">
-        <v>489</v>
+        <v>548</v>
       </c>
     </row>
     <row r="190" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -10954,7 +10954,7 @@
         <v>60</v>
       </c>
       <c r="I190" s="19">
-        <v>306</v>
+        <v>348</v>
       </c>
     </row>
     <row r="191" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -10983,7 +10983,7 @@
         <v>51</v>
       </c>
       <c r="I191" s="19">
-        <v>688</v>
+        <v>523</v>
       </c>
     </row>
     <row r="192" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -11012,7 +11012,7 @@
         <v>51</v>
       </c>
       <c r="I192" s="19">
-        <v>295</v>
+        <v>447</v>
       </c>
     </row>
     <row r="193" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -11041,7 +11041,7 @@
         <v>60</v>
       </c>
       <c r="I193" s="19">
-        <v>323</v>
+        <v>445</v>
       </c>
     </row>
     <row r="194" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -11070,7 +11070,7 @@
         <v>51</v>
       </c>
       <c r="I194" s="19">
-        <v>308</v>
+        <v>350</v>
       </c>
     </row>
     <row r="195" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -11099,7 +11099,7 @@
         <v>51</v>
       </c>
       <c r="I195" s="19">
-        <v>785</v>
+        <v>790</v>
       </c>
     </row>
     <row r="196" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -11128,7 +11128,7 @@
         <v>60</v>
       </c>
       <c r="I196" s="19">
-        <v>581</v>
+        <v>715</v>
       </c>
     </row>
     <row r="197" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -11157,7 +11157,7 @@
         <v>51</v>
       </c>
       <c r="I197" s="19">
-        <v>238</v>
+        <v>637</v>
       </c>
     </row>
     <row r="198" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -11186,7 +11186,7 @@
         <v>51</v>
       </c>
       <c r="I198" s="19">
-        <v>521</v>
+        <v>454</v>
       </c>
     </row>
     <row r="199" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -11215,7 +11215,7 @@
         <v>60</v>
       </c>
       <c r="I199" s="19">
-        <v>440</v>
+        <v>692</v>
       </c>
     </row>
     <row r="200" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -11244,7 +11244,7 @@
         <v>51</v>
       </c>
       <c r="I200" s="19">
-        <v>681</v>
+        <v>397</v>
       </c>
     </row>
     <row r="201" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -11273,7 +11273,7 @@
         <v>51</v>
       </c>
       <c r="I201" s="19">
-        <v>655</v>
+        <v>304</v>
       </c>
     </row>
     <row r="202" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -11302,7 +11302,7 @@
         <v>60</v>
       </c>
       <c r="I202" s="19">
-        <v>329</v>
+        <v>644</v>
       </c>
     </row>
     <row r="203" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -11331,7 +11331,7 @@
         <v>51</v>
       </c>
       <c r="I203" s="19">
-        <v>602</v>
+        <v>322</v>
       </c>
     </row>
     <row r="204" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -11360,7 +11360,7 @@
         <v>51</v>
       </c>
       <c r="I204" s="19">
-        <v>295</v>
+        <v>411</v>
       </c>
     </row>
     <row r="205" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -11389,7 +11389,7 @@
         <v>60</v>
       </c>
       <c r="I205" s="19">
-        <v>780</v>
+        <v>276</v>
       </c>
     </row>
     <row r="206" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -11418,7 +11418,7 @@
         <v>51</v>
       </c>
       <c r="I206" s="19">
-        <v>496</v>
+        <v>758</v>
       </c>
     </row>
     <row r="207" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -11447,7 +11447,7 @@
         <v>51</v>
       </c>
       <c r="I207" s="19">
-        <v>223</v>
+        <v>270</v>
       </c>
     </row>
     <row r="208" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -11476,7 +11476,7 @@
         <v>60</v>
       </c>
       <c r="I208" s="19">
-        <v>400</v>
+        <v>216</v>
       </c>
     </row>
     <row r="209" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -11505,7 +11505,7 @@
         <v>51</v>
       </c>
       <c r="I209" s="19">
-        <v>482</v>
+        <v>690</v>
       </c>
     </row>
     <row r="210" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -11534,7 +11534,7 @@
         <v>51</v>
       </c>
       <c r="I210" s="19">
-        <v>211</v>
+        <v>351</v>
       </c>
     </row>
     <row r="211" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -11563,7 +11563,7 @@
         <v>60</v>
       </c>
       <c r="I211" s="19">
-        <v>679</v>
+        <v>597</v>
       </c>
     </row>
     <row r="212" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -11592,7 +11592,7 @@
         <v>51</v>
       </c>
       <c r="I212" s="19">
-        <v>539</v>
+        <v>534</v>
       </c>
     </row>
     <row r="213" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -11621,7 +11621,7 @@
         <v>51</v>
       </c>
       <c r="I213" s="19">
-        <v>588</v>
+        <v>258</v>
       </c>
     </row>
     <row r="214" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -11650,7 +11650,7 @@
         <v>60</v>
       </c>
       <c r="I214" s="19">
-        <v>635</v>
+        <v>626</v>
       </c>
     </row>
     <row r="215" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -11679,7 +11679,7 @@
         <v>51</v>
       </c>
       <c r="I215" s="19">
-        <v>533</v>
+        <v>709</v>
       </c>
     </row>
     <row r="216" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -11708,7 +11708,7 @@
         <v>51</v>
       </c>
       <c r="I216" s="19">
-        <v>644</v>
+        <v>338</v>
       </c>
     </row>
     <row r="217" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -11737,7 +11737,7 @@
         <v>60</v>
       </c>
       <c r="I217" s="19">
-        <v>702</v>
+        <v>409</v>
       </c>
     </row>
     <row r="218" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -11766,7 +11766,7 @@
         <v>51</v>
       </c>
       <c r="I218" s="19">
-        <v>301</v>
+        <v>414</v>
       </c>
     </row>
     <row r="219" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -11795,7 +11795,7 @@
         <v>51</v>
       </c>
       <c r="I219" s="19">
-        <v>268</v>
+        <v>520</v>
       </c>
     </row>
     <row r="220" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -11824,7 +11824,7 @@
         <v>60</v>
       </c>
       <c r="I220" s="19">
-        <v>556</v>
+        <v>280</v>
       </c>
     </row>
     <row r="221" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -11853,7 +11853,7 @@
         <v>51</v>
       </c>
       <c r="I221" s="19">
-        <v>400</v>
+        <v>768</v>
       </c>
     </row>
     <row r="222" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -11882,7 +11882,7 @@
         <v>51</v>
       </c>
       <c r="I222" s="19">
-        <v>576</v>
+        <v>301</v>
       </c>
     </row>
     <row r="223" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -11911,7 +11911,7 @@
         <v>60</v>
       </c>
       <c r="I223" s="19">
-        <v>717</v>
+        <v>287</v>
       </c>
     </row>
     <row r="224" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -11940,7 +11940,7 @@
         <v>51</v>
       </c>
       <c r="I224" s="19">
-        <v>350</v>
+        <v>575</v>
       </c>
     </row>
     <row r="225" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -11969,7 +11969,7 @@
         <v>51</v>
       </c>
       <c r="I225" s="19">
-        <v>411</v>
+        <v>310</v>
       </c>
     </row>
     <row r="226" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -11998,7 +11998,7 @@
         <v>60</v>
       </c>
       <c r="I226" s="19">
-        <v>451</v>
+        <v>666</v>
       </c>
     </row>
     <row r="227" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -12027,7 +12027,7 @@
         <v>51</v>
       </c>
       <c r="I227" s="19">
-        <v>550</v>
+        <v>613</v>
       </c>
     </row>
     <row r="228" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -12056,7 +12056,7 @@
         <v>51</v>
       </c>
       <c r="I228" s="19">
-        <v>356</v>
+        <v>345</v>
       </c>
     </row>
     <row r="229" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -12085,7 +12085,7 @@
         <v>60</v>
       </c>
       <c r="I229" s="19">
-        <v>271</v>
+        <v>657</v>
       </c>
     </row>
     <row r="230" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -12114,7 +12114,7 @@
         <v>51</v>
       </c>
       <c r="I230" s="19">
-        <v>630</v>
+        <v>607</v>
       </c>
     </row>
     <row r="231" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -12143,7 +12143,7 @@
         <v>51</v>
       </c>
       <c r="I231" s="19">
-        <v>290</v>
+        <v>347</v>
       </c>
     </row>
     <row r="232" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -12172,7 +12172,7 @@
         <v>60</v>
       </c>
       <c r="I232" s="19">
-        <v>583</v>
+        <v>470</v>
       </c>
     </row>
     <row r="233" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -12201,7 +12201,7 @@
         <v>51</v>
       </c>
       <c r="I233" s="19">
-        <v>613</v>
+        <v>306</v>
       </c>
     </row>
     <row r="234" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -12230,7 +12230,7 @@
         <v>51</v>
       </c>
       <c r="I234" s="19">
-        <v>616</v>
+        <v>344</v>
       </c>
     </row>
     <row r="235" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -12259,7 +12259,7 @@
         <v>60</v>
       </c>
       <c r="I235" s="19">
-        <v>201</v>
+        <v>317</v>
       </c>
     </row>
     <row r="236" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -12288,7 +12288,7 @@
         <v>51</v>
       </c>
       <c r="I236" s="19">
-        <v>535</v>
+        <v>267</v>
       </c>
     </row>
     <row r="237" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -12317,7 +12317,7 @@
         <v>51</v>
       </c>
       <c r="I237" s="19">
-        <v>714</v>
+        <v>775</v>
       </c>
     </row>
     <row r="238" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -12346,7 +12346,7 @@
         <v>60</v>
       </c>
       <c r="I238" s="19">
-        <v>774</v>
+        <v>211</v>
       </c>
     </row>
     <row r="239" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -12375,7 +12375,7 @@
         <v>51</v>
       </c>
       <c r="I239" s="19">
-        <v>626</v>
+        <v>449</v>
       </c>
     </row>
     <row r="240" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -12404,7 +12404,7 @@
         <v>51</v>
       </c>
       <c r="I240" s="19">
-        <v>777</v>
+        <v>435</v>
       </c>
     </row>
     <row r="241" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -12433,7 +12433,7 @@
         <v>292</v>
       </c>
       <c r="I241" s="19">
-        <v>386</v>
+        <v>350</v>
       </c>
     </row>
     <row r="242" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -12462,7 +12462,7 @@
         <v>51</v>
       </c>
       <c r="I242" s="19">
-        <v>299</v>
+        <v>422</v>
       </c>
     </row>
     <row r="243" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -12491,7 +12491,7 @@
         <v>51</v>
       </c>
       <c r="I243" s="19">
-        <v>278</v>
+        <v>528</v>
       </c>
     </row>
     <row r="244" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -12520,7 +12520,7 @@
         <v>60</v>
       </c>
       <c r="I244" s="19">
-        <v>548</v>
+        <v>299</v>
       </c>
     </row>
     <row r="245" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -12549,7 +12549,7 @@
         <v>51</v>
       </c>
       <c r="I245" s="19">
-        <v>744</v>
+        <v>475</v>
       </c>
     </row>
     <row r="246" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -12578,7 +12578,7 @@
         <v>51</v>
       </c>
       <c r="I246" s="19">
-        <v>404</v>
+        <v>651</v>
       </c>
     </row>
     <row r="247" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -12607,7 +12607,7 @@
         <v>60</v>
       </c>
       <c r="I247" s="19">
-        <v>720</v>
+        <v>417</v>
       </c>
     </row>
     <row r="248" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -12636,7 +12636,7 @@
         <v>51</v>
       </c>
       <c r="I248" s="19">
-        <v>743</v>
+        <v>278</v>
       </c>
     </row>
     <row r="249" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -12665,7 +12665,7 @@
         <v>51</v>
       </c>
       <c r="I249" s="19">
-        <v>445</v>
+        <v>705</v>
       </c>
     </row>
     <row r="250" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -12694,7 +12694,7 @@
         <v>60</v>
       </c>
       <c r="I250" s="19">
-        <v>263</v>
+        <v>445</v>
       </c>
     </row>
     <row r="251" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -12723,7 +12723,7 @@
         <v>51</v>
       </c>
       <c r="I251" s="19">
-        <v>461</v>
+        <v>431</v>
       </c>
     </row>
     <row r="252" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -12752,7 +12752,7 @@
         <v>51</v>
       </c>
       <c r="I252" s="19">
-        <v>645</v>
+        <v>238</v>
       </c>
     </row>
     <row r="253" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -12781,7 +12781,7 @@
         <v>60</v>
       </c>
       <c r="I253" s="19">
-        <v>645</v>
+        <v>579</v>
       </c>
     </row>
     <row r="254" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -12810,7 +12810,7 @@
         <v>51</v>
       </c>
       <c r="I254" s="19">
-        <v>730</v>
+        <v>306</v>
       </c>
     </row>
     <row r="255" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -12839,7 +12839,7 @@
         <v>51</v>
       </c>
       <c r="I255" s="19">
-        <v>223</v>
+        <v>610</v>
       </c>
     </row>
     <row r="256" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -12868,7 +12868,7 @@
         <v>60</v>
       </c>
       <c r="I256" s="19">
-        <v>236</v>
+        <v>442</v>
       </c>
     </row>
     <row r="257" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -12897,7 +12897,7 @@
         <v>51</v>
       </c>
       <c r="I257" s="19">
-        <v>500</v>
+        <v>277</v>
       </c>
     </row>
     <row r="258" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -12926,7 +12926,7 @@
         <v>51</v>
       </c>
       <c r="I258" s="19">
-        <v>246</v>
+        <v>499</v>
       </c>
     </row>
     <row r="259" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -12955,7 +12955,7 @@
         <v>60</v>
       </c>
       <c r="I259" s="19">
-        <v>234</v>
+        <v>684</v>
       </c>
     </row>
     <row r="260" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -12984,7 +12984,7 @@
         <v>51</v>
       </c>
       <c r="I260" s="19">
-        <v>449</v>
+        <v>318</v>
       </c>
     </row>
     <row r="261" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -13013,7 +13013,7 @@
         <v>51</v>
       </c>
       <c r="I261" s="19">
-        <v>271</v>
+        <v>697</v>
       </c>
     </row>
     <row r="262" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -13042,7 +13042,7 @@
         <v>60</v>
       </c>
       <c r="I262" s="19">
-        <v>624</v>
+        <v>372</v>
       </c>
     </row>
     <row r="263" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -13071,7 +13071,7 @@
         <v>51</v>
       </c>
       <c r="I263" s="19">
-        <v>592</v>
+        <v>366</v>
       </c>
     </row>
     <row r="264" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -13100,7 +13100,7 @@
         <v>51</v>
       </c>
       <c r="I264" s="19">
-        <v>657</v>
+        <v>688</v>
       </c>
     </row>
     <row r="265" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -13129,7 +13129,7 @@
         <v>60</v>
       </c>
       <c r="I265" s="19">
-        <v>343</v>
+        <v>299</v>
       </c>
     </row>
     <row r="266" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -13158,7 +13158,7 @@
         <v>51</v>
       </c>
       <c r="I266" s="19">
-        <v>750</v>
+        <v>263</v>
       </c>
     </row>
     <row r="267" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -13187,7 +13187,7 @@
         <v>51</v>
       </c>
       <c r="I267" s="19">
-        <v>455</v>
+        <v>784</v>
       </c>
     </row>
     <row r="268" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -13216,7 +13216,7 @@
         <v>60</v>
       </c>
       <c r="I268" s="19">
-        <v>626</v>
+        <v>465</v>
       </c>
     </row>
     <row r="269" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -13245,7 +13245,7 @@
         <v>51</v>
       </c>
       <c r="I269" s="19">
-        <v>251</v>
+        <v>370</v>
       </c>
     </row>
     <row r="270" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -13274,7 +13274,7 @@
         <v>51</v>
       </c>
       <c r="I270" s="19">
-        <v>367</v>
+        <v>786</v>
       </c>
     </row>
     <row r="271" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -13303,7 +13303,7 @@
         <v>60</v>
       </c>
       <c r="I271" s="19">
-        <v>750</v>
+        <v>423</v>
       </c>
     </row>
     <row r="272" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -13332,7 +13332,7 @@
         <v>51</v>
       </c>
       <c r="I272" s="19">
-        <v>542</v>
+        <v>759</v>
       </c>
     </row>
     <row r="273" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -13361,7 +13361,7 @@
         <v>51</v>
       </c>
       <c r="I273" s="19">
-        <v>373</v>
+        <v>719</v>
       </c>
     </row>
     <row r="274" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -13390,7 +13390,7 @@
         <v>60</v>
       </c>
       <c r="I274" s="19">
-        <v>587</v>
+        <v>693</v>
       </c>
     </row>
     <row r="275" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -13419,7 +13419,7 @@
         <v>51</v>
       </c>
       <c r="I275" s="19">
-        <v>432</v>
+        <v>388</v>
       </c>
     </row>
     <row r="276" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -13448,7 +13448,7 @@
         <v>51</v>
       </c>
       <c r="I276" s="19">
-        <v>705</v>
+        <v>770</v>
       </c>
     </row>
     <row r="277" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -13477,7 +13477,7 @@
         <v>60</v>
       </c>
       <c r="I277" s="19">
-        <v>791</v>
+        <v>426</v>
       </c>
     </row>
     <row r="278" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -13506,7 +13506,7 @@
         <v>51</v>
       </c>
       <c r="I278" s="19">
-        <v>697</v>
+        <v>321</v>
       </c>
     </row>
     <row r="279" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -13535,7 +13535,7 @@
         <v>51</v>
       </c>
       <c r="I279" s="19">
-        <v>354</v>
+        <v>315</v>
       </c>
     </row>
     <row r="280" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -13564,7 +13564,7 @@
         <v>60</v>
       </c>
       <c r="I280" s="19">
-        <v>368</v>
+        <v>350</v>
       </c>
     </row>
     <row r="281" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -13593,7 +13593,7 @@
         <v>51</v>
       </c>
       <c r="I281" s="19">
-        <v>379</v>
+        <v>324</v>
       </c>
     </row>
     <row r="282" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -13622,7 +13622,7 @@
         <v>51</v>
       </c>
       <c r="I282" s="19">
-        <v>590</v>
+        <v>366</v>
       </c>
     </row>
     <row r="283" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -13651,7 +13651,7 @@
         <v>60</v>
       </c>
       <c r="I283" s="19">
-        <v>290</v>
+        <v>453</v>
       </c>
     </row>
     <row r="284" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -13680,7 +13680,7 @@
         <v>51</v>
       </c>
       <c r="I284" s="19">
-        <v>770</v>
+        <v>584</v>
       </c>
     </row>
     <row r="285" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -13709,7 +13709,7 @@
         <v>51</v>
       </c>
       <c r="I285" s="19">
-        <v>775</v>
+        <v>798</v>
       </c>
     </row>
     <row r="286" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -13738,7 +13738,7 @@
         <v>60</v>
       </c>
       <c r="I286" s="19">
-        <v>582</v>
+        <v>669</v>
       </c>
     </row>
     <row r="287" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -13767,7 +13767,7 @@
         <v>51</v>
       </c>
       <c r="I287" s="19">
-        <v>335</v>
+        <v>255</v>
       </c>
     </row>
     <row r="288" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -13796,7 +13796,7 @@
         <v>51</v>
       </c>
       <c r="I288" s="19">
-        <v>701</v>
+        <v>529</v>
       </c>
     </row>
     <row r="289" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -13825,7 +13825,7 @@
         <v>60</v>
       </c>
       <c r="I289" s="19">
-        <v>271</v>
+        <v>318</v>
       </c>
     </row>
     <row r="290" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -13854,7 +13854,7 @@
         <v>51</v>
       </c>
       <c r="I290" s="19">
-        <v>236</v>
+        <v>609</v>
       </c>
     </row>
     <row r="291" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -13883,7 +13883,7 @@
         <v>51</v>
       </c>
       <c r="I291" s="19">
-        <v>614</v>
+        <v>535</v>
       </c>
     </row>
     <row r="292" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -13912,7 +13912,7 @@
         <v>60</v>
       </c>
       <c r="I292" s="19">
-        <v>778</v>
+        <v>715</v>
       </c>
     </row>
     <row r="293" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -13941,7 +13941,7 @@
         <v>51</v>
       </c>
       <c r="I293" s="19">
-        <v>389</v>
+        <v>335</v>
       </c>
     </row>
     <row r="294" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -13970,7 +13970,7 @@
         <v>51</v>
       </c>
       <c r="I294" s="19">
-        <v>550</v>
+        <v>475</v>
       </c>
     </row>
     <row r="295" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -13999,7 +13999,7 @@
         <v>60</v>
       </c>
       <c r="I295" s="19">
-        <v>778</v>
+        <v>430</v>
       </c>
     </row>
     <row r="296" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -14028,7 +14028,7 @@
         <v>51</v>
       </c>
       <c r="I296" s="19">
-        <v>444</v>
+        <v>681</v>
       </c>
     </row>
     <row r="297" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -14057,7 +14057,7 @@
         <v>51</v>
       </c>
       <c r="I297" s="19">
-        <v>382</v>
+        <v>719</v>
       </c>
     </row>
     <row r="298" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -14086,7 +14086,7 @@
         <v>60</v>
       </c>
       <c r="I298" s="19">
-        <v>418</v>
+        <v>618</v>
       </c>
     </row>
     <row r="299" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -14115,7 +14115,7 @@
         <v>51</v>
       </c>
       <c r="I299" s="19">
-        <v>212</v>
+        <v>659</v>
       </c>
     </row>
     <row r="300" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -14144,7 +14144,7 @@
         <v>51</v>
       </c>
       <c r="I300" s="19">
-        <v>363</v>
+        <v>565</v>
       </c>
     </row>
     <row r="301" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -14173,7 +14173,7 @@
         <v>292</v>
       </c>
       <c r="I301" s="19">
-        <v>396</v>
+        <v>309</v>
       </c>
     </row>
     <row r="302" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -14202,7 +14202,7 @@
         <v>51</v>
       </c>
       <c r="I302" s="19">
-        <v>445</v>
+        <v>312</v>
       </c>
     </row>
     <row r="303" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -14231,7 +14231,7 @@
         <v>51</v>
       </c>
       <c r="I303" s="19">
-        <v>512</v>
+        <v>453</v>
       </c>
     </row>
     <row r="304" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -14260,7 +14260,7 @@
         <v>60</v>
       </c>
       <c r="I304" s="19">
-        <v>765</v>
+        <v>480</v>
       </c>
     </row>
     <row r="305" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -14289,7 +14289,7 @@
         <v>51</v>
       </c>
       <c r="I305" s="19">
-        <v>395</v>
+        <v>716</v>
       </c>
     </row>
     <row r="306" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -14318,7 +14318,7 @@
         <v>51</v>
       </c>
       <c r="I306" s="19">
-        <v>346</v>
+        <v>329</v>
       </c>
     </row>
     <row r="307" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -14347,7 +14347,7 @@
         <v>60</v>
       </c>
       <c r="I307" s="19">
-        <v>541</v>
+        <v>714</v>
       </c>
     </row>
     <row r="308" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -14376,7 +14376,7 @@
         <v>51</v>
       </c>
       <c r="I308" s="19">
-        <v>562</v>
+        <v>400</v>
       </c>
     </row>
     <row r="309" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -14405,7 +14405,7 @@
         <v>51</v>
       </c>
       <c r="I309" s="19">
-        <v>326</v>
+        <v>346</v>
       </c>
     </row>
     <row r="310" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -14434,7 +14434,7 @@
         <v>60</v>
       </c>
       <c r="I310" s="19">
-        <v>274</v>
+        <v>331</v>
       </c>
     </row>
     <row r="311" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -14463,7 +14463,7 @@
         <v>51</v>
       </c>
       <c r="I311" s="19">
-        <v>699</v>
+        <v>204</v>
       </c>
     </row>
   </sheetData>

</xml_diff>